<commit_message>
Cleanup commit before refresh
</commit_message>
<xml_diff>
--- a/TestCases/AllTestcaseSuite.xlsx
+++ b/TestCases/AllTestcaseSuite.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -935,25 +935,25 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>test_API_SA_PreFetch_01</t>
+          <t>test_success_2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Functional/API_DB/SA/test_API_SA_PreFetch</t>
+          <t>test_sample</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>API_DB/SA</t>
+          <t>UI/SA</t>
         </is>
       </c>
       <c r="E23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -962,17 +962,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>test_GUI_APP_Branding_Ezetap_01</t>
+          <t>test_API_SA_PreFetch_01</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GUI/APP/test_GUI_APP_Branding</t>
+          <t>Functional/API_DB/SA/test_API_SA_PreFetch</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>GUI/APP</t>
+          <t>API_DB/SA</t>
         </is>
       </c>
       <c r="E24" t="b">
@@ -981,11 +981,11 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>test_GUI_APP_Branding_Axis_02</t>
+          <t>test_GUI_APP_Branding_Ezetap_01</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1004,24 +1004,47 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>test_GUI_APP_Branding_Axis_02</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>GUI/APP/test_GUI_APP_Branding</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>GUI/APP</t>
+        </is>
+      </c>
+      <c r="E26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>test_GUI_APP_Branding_Hdfc_03</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>GUI/APP/test_GUI_APP_Branding</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>GUI/APP</t>
         </is>
       </c>
-      <c r="E26" t="b">
+      <c r="E27" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>